<commit_message>
Update Trading Journal.xlsx 2026-09-25 10:38:29
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -429,7 +429,8 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,6 +471,11 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>零股(股)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
@@ -507,6 +513,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="1" t="inlineStr"/>
+      <c r="I2" s="1" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -541,6 +548,7 @@
         <v>1</v>
       </c>
       <c r="H3" s="1" t="inlineStr"/>
+      <c r="I3" s="1" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -575,6 +583,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="1" t="inlineStr"/>
+      <c r="I4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -609,6 +618,7 @@
         <v>1</v>
       </c>
       <c r="H5" s="1" t="inlineStr"/>
+      <c r="I5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -637,6 +647,7 @@
       <c r="F6" s="1" t="inlineStr"/>
       <c r="G6" s="1" t="inlineStr"/>
       <c r="H6" s="1" t="inlineStr"/>
+      <c r="I6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -665,6 +676,7 @@
       <c r="F7" s="1" t="inlineStr"/>
       <c r="G7" s="1" t="inlineStr"/>
       <c r="H7" s="1" t="inlineStr"/>
+      <c r="I7" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-25 10:47:03
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,15 +419,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="8" customWidth="1" min="9" max="9"/>
@@ -623,21 +623,21 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>00406A</t>
+          <t>4958</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>主動中信台灣收益</t>
+          <t>臻鼎-KY</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>1</v>
+        <v>506</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
@@ -652,21 +652,21 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>4958</t>
+          <t>0050</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>臻鼎-KY</t>
+          <t>元大台灣50</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>506</v>
+        <v>79.52</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
@@ -675,8 +675,173 @@
       </c>
       <c r="F7" s="1" t="inlineStr"/>
       <c r="G7" s="1" t="inlineStr"/>
-      <c r="H7" s="1" t="inlineStr"/>
+      <c r="H7" s="1" t="n">
+        <v>800</v>
+      </c>
       <c r="I7" s="1" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>00981A</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>主動統一台股增長</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>29.64</v>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr"/>
+      <c r="G8" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="1" t="inlineStr"/>
+      <c r="I8" s="1" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>2308</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>台達電</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr"/>
+      <c r="G9" s="1" t="inlineStr"/>
+      <c r="H9" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="I9" s="1" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>2308</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>台達電</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>1890</v>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr"/>
+      <c r="G10" s="1" t="inlineStr"/>
+      <c r="H10" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>2308</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>台達電</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>1900</v>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>下降趨勢線突破</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr"/>
+      <c r="H11" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I11" s="1" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>2317</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>鴻海</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>253</v>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>3K反轉</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr"/>
+      <c r="H12" s="1" t="n">
+        <v>200</v>
+      </c>
+      <c r="I12" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-25 10:52:19
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -842,6 +842,99 @@
         <v>200</v>
       </c>
       <c r="I12" s="1" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>2330</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>台積電</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>1870</v>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr"/>
+      <c r="G13" s="1" t="inlineStr"/>
+      <c r="H13" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="I13" s="1" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>2330</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>台積電</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>2305</v>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr"/>
+      <c r="G14" s="1" t="inlineStr"/>
+      <c r="H14" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="I14" s="1" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>2330</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>台積電</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>2200</v>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr"/>
+      <c r="G15" s="1" t="inlineStr"/>
+      <c r="H15" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="I15" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-25 11:02:30
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -935,6 +935,289 @@
         <v>5</v>
       </c>
       <c r="I15" s="1" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>2357</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>華碩</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>802</v>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr"/>
+      <c r="G16" s="1" t="inlineStr"/>
+      <c r="H16" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="I16" s="1" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>2357</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>華碩</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>917</v>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr"/>
+      <c r="G17" s="1" t="inlineStr"/>
+      <c r="H17" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="I17" s="1" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>2025-11-21</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>2383</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>台光電</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>1320</v>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr"/>
+      <c r="G18" s="1" t="inlineStr"/>
+      <c r="H18" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="I18" s="1" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>2454</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>聯發科</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>4160</v>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr"/>
+      <c r="G19" s="1" t="inlineStr"/>
+      <c r="H19" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="I19" s="1" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>大立光</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>2565</v>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr"/>
+      <c r="G20" s="1" t="inlineStr"/>
+      <c r="H20" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="I20" s="1" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>3008</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>大立光</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>4050</v>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr"/>
+      <c r="G21" s="1" t="inlineStr"/>
+      <c r="H21" s="1" t="n">
+        <v>25</v>
+      </c>
+      <c r="I21" s="1" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>3081</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>聯亞</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>2775</v>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr"/>
+      <c r="H22" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="I22" s="1" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>3711</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>日月光投控</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>680</v>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr"/>
+      <c r="G23" s="1" t="inlineStr"/>
+      <c r="H23" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I23" s="1" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>3711</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>日月光投控</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>624</v>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr"/>
+      <c r="G24" s="1" t="inlineStr"/>
+      <c r="H24" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="I24" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-25 11:14:19
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1218,6 +1218,324 @@
         <v>50</v>
       </c>
       <c r="I24" s="1" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>4958</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>臻鼎-KY</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>438.5</v>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr"/>
+      <c r="G25" s="1" t="inlineStr"/>
+      <c r="H25" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="I25" s="1" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr">
+        <is>
+          <t>4958</t>
+        </is>
+      </c>
+      <c r="C26" s="1" t="inlineStr">
+        <is>
+          <t>臻鼎-KY</t>
+        </is>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>506</v>
+      </c>
+      <c r="E26" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F26" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr"/>
+      <c r="H26" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="I26" s="1" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>5443</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>均豪</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>115.5</v>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr"/>
+      <c r="G27" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="1" t="inlineStr"/>
+      <c r="I27" s="1" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>5443</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
+        <is>
+          <t>均豪</t>
+        </is>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>108</v>
+      </c>
+      <c r="E28" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F28" s="1" t="inlineStr"/>
+      <c r="G28" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="1" t="inlineStr"/>
+      <c r="I28" s="1" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>6015</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
+        <is>
+          <t>宏遠證</t>
+        </is>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>18.88</v>
+      </c>
+      <c r="E29" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F29" s="1" t="inlineStr"/>
+      <c r="G29" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="1" t="inlineStr"/>
+      <c r="I29" s="1" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>6147</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
+        <is>
+          <t>頎邦</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>184</v>
+      </c>
+      <c r="E30" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F30" s="1" t="inlineStr"/>
+      <c r="G30" s="1" t="inlineStr"/>
+      <c r="H30" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="I30" s="1" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>6147</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
+        <is>
+          <t>頎邦</t>
+        </is>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>192.5</v>
+      </c>
+      <c r="E31" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F31" s="1" t="inlineStr"/>
+      <c r="G31" s="1" t="inlineStr"/>
+      <c r="H31" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="I31" s="1" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>6147</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>頎邦</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>227</v>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr"/>
+      <c r="G32" s="1" t="inlineStr"/>
+      <c r="H32" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="I32" s="1" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>6147</t>
+        </is>
+      </c>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>頎邦</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>224.5</v>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr"/>
+      <c r="G33" s="1" t="inlineStr"/>
+      <c r="H33" s="1" t="n">
+        <v>250</v>
+      </c>
+      <c r="I33" s="1" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>8064</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>東捷</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>133.5</v>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G34" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="1" t="inlineStr"/>
+      <c r="I34" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-25 11:19:04
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -623,21 +623,21 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>4958</t>
+          <t>0050</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>臻鼎-KY</t>
+          <t>元大台灣50</t>
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>506</v>
+        <v>79.52</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
@@ -646,27 +646,29 @@
       </c>
       <c r="F6" s="1" t="inlineStr"/>
       <c r="G6" s="1" t="inlineStr"/>
-      <c r="H6" s="1" t="inlineStr"/>
+      <c r="H6" s="1" t="n">
+        <v>800</v>
+      </c>
       <c r="I6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>0050</t>
+          <t>00981A</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>元大台灣50</t>
+          <t>主動統一台股增長</t>
         </is>
       </c>
       <c r="D7" s="1" t="n">
-        <v>79.52</v>
+        <v>29.64</v>
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
@@ -674,30 +676,30 @@
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr"/>
-      <c r="G7" s="1" t="inlineStr"/>
-      <c r="H7" s="1" t="n">
-        <v>800</v>
-      </c>
+      <c r="G7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="1" t="inlineStr"/>
       <c r="I7" s="1" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>00981A</t>
+          <t>2308</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>主動統一台股增長</t>
+          <t>台達電</t>
         </is>
       </c>
       <c r="D8" s="1" t="n">
-        <v>29.64</v>
+        <v>2015</v>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
@@ -705,16 +707,16 @@
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr"/>
-      <c r="G8" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" s="1" t="inlineStr"/>
+      <c r="G8" s="1" t="inlineStr"/>
+      <c r="H8" s="1" t="n">
+        <v>40</v>
+      </c>
       <c r="I8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B9" s="1" t="inlineStr">
@@ -728,7 +730,7 @@
         </is>
       </c>
       <c r="D9" s="1" t="n">
-        <v>2015</v>
+        <v>1890</v>
       </c>
       <c r="E9" s="1" t="inlineStr">
         <is>
@@ -738,14 +740,14 @@
       <c r="F9" s="1" t="inlineStr"/>
       <c r="G9" s="1" t="inlineStr"/>
       <c r="H9" s="1" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="I9" s="1" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
@@ -759,14 +761,18 @@
         </is>
       </c>
       <c r="D10" s="1" t="n">
-        <v>1890</v>
+        <v>1900</v>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
           <t>買入</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr"/>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>下降趨勢線突破</t>
+        </is>
+      </c>
       <c r="G10" s="1" t="inlineStr"/>
       <c r="H10" s="1" t="n">
         <v>10</v>
@@ -781,16 +787,16 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>2308</t>
+          <t>2317</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>台達電</t>
+          <t>鴻海</t>
         </is>
       </c>
       <c r="D11" s="1" t="n">
-        <v>1900</v>
+        <v>253</v>
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
@@ -799,54 +805,50 @@
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>下降趨勢線突破</t>
+          <t>3K反轉</t>
         </is>
       </c>
       <c r="G11" s="1" t="inlineStr"/>
       <c r="H11" s="1" t="n">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="I11" s="1" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>2317</t>
+          <t>2330</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>鴻海</t>
+          <t>台積電</t>
         </is>
       </c>
       <c r="D12" s="1" t="n">
-        <v>253</v>
+        <v>1870</v>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
           <t>買入</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>3K反轉</t>
-        </is>
-      </c>
+      <c r="F12" s="1" t="inlineStr"/>
       <c r="G12" s="1" t="inlineStr"/>
       <c r="H12" s="1" t="n">
-        <v>200</v>
+        <v>55</v>
       </c>
       <c r="I12" s="1" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B13" s="1" t="inlineStr">
@@ -860,7 +862,7 @@
         </is>
       </c>
       <c r="D13" s="1" t="n">
-        <v>1870</v>
+        <v>2305</v>
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
@@ -870,14 +872,14 @@
       <c r="F13" s="1" t="inlineStr"/>
       <c r="G13" s="1" t="inlineStr"/>
       <c r="H13" s="1" t="n">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="I13" s="1" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B14" s="1" t="inlineStr">
@@ -891,7 +893,7 @@
         </is>
       </c>
       <c r="D14" s="1" t="n">
-        <v>2305</v>
+        <v>2200</v>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
@@ -908,21 +910,21 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>2330</t>
+          <t>2357</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>台積電</t>
+          <t>華碩</t>
         </is>
       </c>
       <c r="D15" s="1" t="n">
-        <v>2200</v>
+        <v>802</v>
       </c>
       <c r="E15" s="1" t="inlineStr">
         <is>
@@ -932,14 +934,14 @@
       <c r="F15" s="1" t="inlineStr"/>
       <c r="G15" s="1" t="inlineStr"/>
       <c r="H15" s="1" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="I15" s="1" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B16" s="1" t="inlineStr">
@@ -953,7 +955,7 @@
         </is>
       </c>
       <c r="D16" s="1" t="n">
-        <v>802</v>
+        <v>917</v>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
@@ -970,21 +972,21 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2025-11-21</t>
         </is>
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>2357</t>
+          <t>2383</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>華碩</t>
+          <t>台光電</t>
         </is>
       </c>
       <c r="D17" s="1" t="n">
-        <v>917</v>
+        <v>1320</v>
       </c>
       <c r="E17" s="1" t="inlineStr">
         <is>
@@ -994,28 +996,28 @@
       <c r="F17" s="1" t="inlineStr"/>
       <c r="G17" s="1" t="inlineStr"/>
       <c r="H17" s="1" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="I17" s="1" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>2383</t>
+          <t>2454</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>台光電</t>
+          <t>聯發科</t>
         </is>
       </c>
       <c r="D18" s="1" t="n">
-        <v>1320</v>
+        <v>4160</v>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
@@ -1025,28 +1027,28 @@
       <c r="F18" s="1" t="inlineStr"/>
       <c r="G18" s="1" t="inlineStr"/>
       <c r="H18" s="1" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="I18" s="1" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>2454</t>
+          <t>3008</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>聯發科</t>
+          <t>大立光</t>
         </is>
       </c>
       <c r="D19" s="1" t="n">
-        <v>4160</v>
+        <v>2565</v>
       </c>
       <c r="E19" s="1" t="inlineStr">
         <is>
@@ -1056,14 +1058,14 @@
       <c r="F19" s="1" t="inlineStr"/>
       <c r="G19" s="1" t="inlineStr"/>
       <c r="H19" s="1" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="I19" s="1" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B20" s="1" t="inlineStr">
@@ -1077,7 +1079,7 @@
         </is>
       </c>
       <c r="D20" s="1" t="n">
-        <v>2565</v>
+        <v>4050</v>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
@@ -1087,80 +1089,80 @@
       <c r="F20" s="1" t="inlineStr"/>
       <c r="G20" s="1" t="inlineStr"/>
       <c r="H20" s="1" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="I20" s="1" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>3081</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>大立光</t>
+          <t>聯亞</t>
         </is>
       </c>
       <c r="D21" s="1" t="n">
-        <v>4050</v>
+        <v>2775</v>
       </c>
       <c r="E21" s="1" t="inlineStr">
         <is>
           <t>買入</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr"/>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
       <c r="G21" s="1" t="inlineStr"/>
       <c r="H21" s="1" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="I21" s="1" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>3081</t>
+          <t>3711</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>聯亞</t>
+          <t>日月光投控</t>
         </is>
       </c>
       <c r="D22" s="1" t="n">
-        <v>2775</v>
+        <v>680</v>
       </c>
       <c r="E22" s="1" t="inlineStr">
         <is>
           <t>買入</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
-        <is>
-          <t>巧妙點</t>
-        </is>
-      </c>
+      <c r="F22" s="1" t="inlineStr"/>
       <c r="G22" s="1" t="inlineStr"/>
       <c r="H22" s="1" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="I22" s="1" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B23" s="1" t="inlineStr">
@@ -1174,7 +1176,7 @@
         </is>
       </c>
       <c r="D23" s="1" t="n">
-        <v>680</v>
+        <v>624</v>
       </c>
       <c r="E23" s="1" t="inlineStr">
         <is>
@@ -1184,28 +1186,28 @@
       <c r="F23" s="1" t="inlineStr"/>
       <c r="G23" s="1" t="inlineStr"/>
       <c r="H23" s="1" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="I23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>3711</t>
+          <t>4958</t>
         </is>
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>日月光投控</t>
+          <t>臻鼎-KY</t>
         </is>
       </c>
       <c r="D24" s="1" t="n">
-        <v>624</v>
+        <v>438.5</v>
       </c>
       <c r="E24" s="1" t="inlineStr">
         <is>
@@ -1215,14 +1217,14 @@
       <c r="F24" s="1" t="inlineStr"/>
       <c r="G24" s="1" t="inlineStr"/>
       <c r="H24" s="1" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="I24" s="1" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B25" s="1" t="inlineStr">
@@ -1236,59 +1238,59 @@
         </is>
       </c>
       <c r="D25" s="1" t="n">
-        <v>438.5</v>
+        <v>506</v>
       </c>
       <c r="E25" s="1" t="inlineStr">
         <is>
           <t>買入</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr"/>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
       <c r="G25" s="1" t="inlineStr"/>
       <c r="H25" s="1" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="I25" s="1" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>4958</t>
+          <t>5443</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>臻鼎-KY</t>
+          <t>均豪</t>
         </is>
       </c>
       <c r="D26" s="1" t="n">
-        <v>506</v>
+        <v>115.5</v>
       </c>
       <c r="E26" s="1" t="inlineStr">
         <is>
           <t>買入</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
-        <is>
-          <t>巧妙點</t>
-        </is>
-      </c>
-      <c r="G26" s="1" t="inlineStr"/>
-      <c r="H26" s="1" t="n">
-        <v>150</v>
-      </c>
+      <c r="F26" s="1" t="inlineStr"/>
+      <c r="G26" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="1" t="inlineStr"/>
       <c r="I26" s="1" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
@@ -1302,7 +1304,7 @@
         </is>
       </c>
       <c r="D27" s="1" t="n">
-        <v>115.5</v>
+        <v>108</v>
       </c>
       <c r="E27" s="1" t="inlineStr">
         <is>
@@ -1319,21 +1321,21 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>5443</t>
+          <t>6015</t>
         </is>
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>均豪</t>
+          <t>宏遠證</t>
         </is>
       </c>
       <c r="D28" s="1" t="n">
-        <v>108</v>
+        <v>18.88</v>
       </c>
       <c r="E28" s="1" t="inlineStr">
         <is>
@@ -1342,7 +1344,7 @@
       </c>
       <c r="F28" s="1" t="inlineStr"/>
       <c r="G28" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H28" s="1" t="inlineStr"/>
       <c r="I28" s="1" t="inlineStr"/>
@@ -1350,21 +1352,21 @@
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>6015</t>
+          <t>6147</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>宏遠證</t>
+          <t>頎邦</t>
         </is>
       </c>
       <c r="D29" s="1" t="n">
-        <v>18.88</v>
+        <v>184</v>
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
@@ -1372,16 +1374,16 @@
         </is>
       </c>
       <c r="F29" s="1" t="inlineStr"/>
-      <c r="G29" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="H29" s="1" t="inlineStr"/>
+      <c r="G29" s="1" t="inlineStr"/>
+      <c r="H29" s="1" t="n">
+        <v>250</v>
+      </c>
       <c r="I29" s="1" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B30" s="1" t="inlineStr">
@@ -1395,7 +1397,7 @@
         </is>
       </c>
       <c r="D30" s="1" t="n">
-        <v>184</v>
+        <v>192.5</v>
       </c>
       <c r="E30" s="1" t="inlineStr">
         <is>
@@ -1412,7 +1414,7 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B31" s="1" t="inlineStr">
@@ -1426,7 +1428,7 @@
         </is>
       </c>
       <c r="D31" s="1" t="n">
-        <v>192.5</v>
+        <v>227</v>
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
@@ -1457,7 +1459,7 @@
         </is>
       </c>
       <c r="D32" s="1" t="n">
-        <v>227</v>
+        <v>224.5</v>
       </c>
       <c r="E32" s="1" t="inlineStr">
         <is>
@@ -1474,68 +1476,103 @@
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>6147</t>
+          <t>8064</t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t>頎邦</t>
+          <t>東捷</t>
         </is>
       </c>
       <c r="D33" s="1" t="n">
-        <v>224.5</v>
+        <v>133.5</v>
       </c>
       <c r="E33" s="1" t="inlineStr">
         <is>
           <t>買入</t>
         </is>
       </c>
-      <c r="F33" s="1" t="inlineStr"/>
-      <c r="G33" s="1" t="inlineStr"/>
-      <c r="H33" s="1" t="n">
-        <v>250</v>
-      </c>
+      <c r="F33" s="1" t="inlineStr">
+        <is>
+          <t>巧妙點</t>
+        </is>
+      </c>
+      <c r="G33" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" s="1" t="inlineStr"/>
       <c r="I33" s="1" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>8064</t>
+          <t>2615</t>
         </is>
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t>東捷</t>
+          <t>萬海</t>
         </is>
       </c>
       <c r="D34" s="1" t="n">
-        <v>133.5</v>
+        <v>117.5</v>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>買入</t>
-        </is>
-      </c>
-      <c r="F34" s="1" t="inlineStr">
-        <is>
-          <t>巧妙點</t>
-        </is>
-      </c>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr"/>
       <c r="G34" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H34" s="1" t="inlineStr"/>
       <c r="I34" s="1" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>2303</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>聯電</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>153</v>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>反向島狀</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="1" t="inlineStr"/>
+      <c r="I35" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update Trading Journal.xlsx 2026-09-25 11:26:07
</commit_message>
<xml_diff>
--- a/Trading Journal.xlsx
+++ b/Trading Journal.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1573,6 +1573,72 @@
       </c>
       <c r="H35" s="1" t="inlineStr"/>
       <c r="I35" s="1" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>3362</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>先進光</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>179</v>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>買入</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr"/>
+      <c r="G36" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="1" t="inlineStr"/>
+      <c r="I36" s="1" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>3362</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>先進光</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>190.5</v>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>賣出</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>上升趨勢線跌破</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="1" t="inlineStr"/>
+      <c r="I37" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>